<commit_message>
Update the T Rows
</commit_message>
<xml_diff>
--- a/assets/list/AD_Master_Data Base Templecurraheen Graveyard Feb23.xlsx
+++ b/assets/list/AD_Master_Data Base Templecurraheen Graveyard Feb23.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Templecurraheen\WorkList_CFAD_22092025\Amalgamate_with_CH_Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Templecurraheen\website\assets\list\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6132D962-7E30-43CC-9975-57619A1F59A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA7D897D-6FA8-4524-B183-300D35AAC493}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="46296" windowHeight="25416" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3723" uniqueCount="1583">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3742" uniqueCount="1594">
   <si>
     <t>Mark</t>
   </si>
@@ -4771,6 +4771,39 @@
   </si>
   <si>
     <t>e25b.jpg</t>
+  </si>
+  <si>
+    <t>t152.jpg</t>
+  </si>
+  <si>
+    <t>t153.jpg</t>
+  </si>
+  <si>
+    <t>t154.jpg</t>
+  </si>
+  <si>
+    <t>t155.jpg</t>
+  </si>
+  <si>
+    <t>Denis Fenton</t>
+  </si>
+  <si>
+    <t>Erected in memory of my grandparents Denis Fenton died 1st April 1967 also his parents and forebears dated back to 1700 interred here His loving wife Margaret Fenton (nee Murphy) died 27th Nov 1980 also her parents and family interred in Kilquane cenetery, Knockraha, Cork.</t>
+  </si>
+  <si>
+    <t>Margaret Fenton</t>
+  </si>
+  <si>
+    <t>Fenton (nee Murphy)</t>
+  </si>
+  <si>
+    <t>Jack</t>
+  </si>
+  <si>
+    <t>Jack Fenton</t>
+  </si>
+  <si>
+    <t>t156.jpg</t>
   </si>
 </sst>
 </file>
@@ -6241,7 +6274,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:V462"/>
+  <dimension ref="A1:V464"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
@@ -16002,13 +16035,13 @@
       </c>
       <c r="C382" s="238"/>
       <c r="D382" s="186" t="s">
-        <v>1231</v>
+        <v>45</v>
       </c>
       <c r="E382" s="186" t="s">
-        <v>34</v>
+        <v>45</v>
       </c>
       <c r="G382" s="30" t="s">
-        <v>1232</v>
+        <v>45</v>
       </c>
     </row>
     <row r="383" spans="2:12" ht="18" customHeight="1">
@@ -16017,13 +16050,13 @@
       </c>
       <c r="C383" s="239"/>
       <c r="D383" s="186" t="s">
-        <v>1231</v>
+        <v>45</v>
       </c>
       <c r="E383" s="186" t="s">
-        <v>62</v>
+        <v>45</v>
       </c>
       <c r="G383" s="30" t="s">
-        <v>1234</v>
+        <v>45</v>
       </c>
     </row>
     <row r="384" spans="2:12" ht="18" customHeight="1">
@@ -16032,118 +16065,121 @@
       </c>
       <c r="C384" s="239"/>
       <c r="D384" s="186" t="s">
-        <v>283</v>
+        <v>45</v>
       </c>
       <c r="E384" s="186" t="s">
-        <v>62</v>
+        <v>45</v>
       </c>
       <c r="G384" s="30" t="s">
-        <v>1236</v>
+        <v>45</v>
       </c>
     </row>
     <row r="385" spans="2:12" ht="18" customHeight="1">
-      <c r="B385" s="239" t="s">
-        <v>1237</v>
-      </c>
-      <c r="C385" s="239"/>
+      <c r="B385" s="238" t="s">
+        <v>1240</v>
+      </c>
+      <c r="C385" s="238"/>
       <c r="D385" s="186" t="s">
-        <v>283</v>
+        <v>1088</v>
       </c>
       <c r="E385" s="186" t="s">
-        <v>1238</v>
-      </c>
-      <c r="F385" s="92">
-        <v>1100</v>
+        <v>32</v>
       </c>
       <c r="G385" s="30" t="s">
-        <v>1239</v>
-      </c>
-      <c r="H385" s="35" t="s">
-        <v>323</v>
+        <v>1241</v>
       </c>
     </row>
     <row r="386" spans="2:12" ht="18" customHeight="1">
       <c r="B386" s="239" t="s">
-        <v>1237</v>
+        <v>1242</v>
       </c>
       <c r="C386" s="239"/>
       <c r="D386" s="186" t="s">
-        <v>283</v>
+        <v>1243</v>
       </c>
       <c r="E386" s="186" t="s">
-        <v>34</v>
-      </c>
-      <c r="F386" s="92">
-        <v>915</v>
+        <v>1244</v>
       </c>
       <c r="G386" s="30" t="s">
-        <v>1210</v>
-      </c>
-      <c r="H386" s="35" t="s">
-        <v>906</v>
+        <v>1245</v>
       </c>
     </row>
     <row r="387" spans="2:12" ht="18" customHeight="1">
-      <c r="B387" s="238" t="s">
-        <v>1240</v>
-      </c>
-      <c r="C387" s="238"/>
+      <c r="B387" s="239" t="s">
+        <v>1246</v>
+      </c>
+      <c r="C387" s="239"/>
       <c r="D387" s="186" t="s">
-        <v>1088</v>
+        <v>45</v>
       </c>
       <c r="E387" s="186" t="s">
-        <v>32</v>
+        <v>45</v>
       </c>
       <c r="G387" s="30" t="s">
-        <v>1241</v>
+        <v>45</v>
       </c>
     </row>
     <row r="388" spans="2:12" ht="18" customHeight="1">
       <c r="B388" s="239" t="s">
-        <v>1242</v>
+        <v>1247</v>
       </c>
       <c r="C388" s="239"/>
       <c r="D388" s="186" t="s">
-        <v>1243</v>
+        <v>1248</v>
       </c>
       <c r="E388" s="186" t="s">
-        <v>1244</v>
+        <v>34</v>
       </c>
       <c r="G388" s="30" t="s">
-        <v>1245</v>
+        <v>1249</v>
+      </c>
+      <c r="I388" s="240" t="s">
+        <v>1583</v>
+      </c>
+      <c r="J388" t="s">
+        <v>1250</v>
       </c>
     </row>
     <row r="389" spans="2:12" ht="18" customHeight="1">
       <c r="B389" s="239" t="s">
-        <v>1246</v>
+        <v>1251</v>
       </c>
       <c r="C389" s="239"/>
       <c r="D389" s="186" t="s">
-        <v>45</v>
+        <v>283</v>
       </c>
       <c r="E389" s="186" t="s">
-        <v>45</v>
+        <v>62</v>
       </c>
       <c r="G389" s="30" t="s">
-        <v>45</v>
+        <v>1236</v>
+      </c>
+      <c r="I389" s="240" t="s">
+        <v>1584</v>
       </c>
     </row>
     <row r="390" spans="2:12" ht="18" customHeight="1">
       <c r="B390" s="239" t="s">
-        <v>1247</v>
+        <v>1251</v>
       </c>
       <c r="C390" s="239"/>
       <c r="D390" s="186" t="s">
-        <v>1248</v>
+        <v>283</v>
       </c>
       <c r="E390" s="186" t="s">
-        <v>34</v>
+        <v>1238</v>
+      </c>
+      <c r="F390" s="92">
+        <v>1100</v>
       </c>
       <c r="G390" s="30" t="s">
-        <v>1249</v>
-      </c>
-      <c r="J390" t="s">
-        <v>1250</v>
+        <v>1239</v>
+      </c>
+      <c r="H390" s="35" t="s">
+        <v>323</v>
+      </c>
+      <c r="I390" s="240" t="s">
+        <v>1584</v>
       </c>
     </row>
     <row r="391" spans="2:12" ht="18" customHeight="1">
@@ -16152,13 +16188,22 @@
       </c>
       <c r="C391" s="239"/>
       <c r="D391" s="186" t="s">
-        <v>45</v>
+        <v>283</v>
       </c>
       <c r="E391" s="186" t="s">
-        <v>45</v>
+        <v>34</v>
+      </c>
+      <c r="F391" s="92">
+        <v>915</v>
       </c>
       <c r="G391" s="30" t="s">
-        <v>1252</v>
+        <v>1210</v>
+      </c>
+      <c r="H391" s="35" t="s">
+        <v>906</v>
+      </c>
+      <c r="I391" s="240" t="s">
+        <v>1584</v>
       </c>
     </row>
     <row r="392" spans="2:12" ht="18" customHeight="1">
@@ -16167,31 +16212,34 @@
       </c>
       <c r="C392" s="239"/>
       <c r="D392" s="186" t="s">
-        <v>45</v>
+        <v>1231</v>
       </c>
       <c r="E392" s="186" t="s">
-        <v>45</v>
+        <v>62</v>
       </c>
       <c r="G392" s="30" t="s">
-        <v>1252</v>
-      </c>
-      <c r="J392" t="s">
-        <v>1254</v>
+        <v>1234</v>
+      </c>
+      <c r="I392" s="240" t="s">
+        <v>1585</v>
       </c>
     </row>
     <row r="393" spans="2:12" ht="18" customHeight="1">
-      <c r="B393" s="239" t="s">
+      <c r="B393" s="238" t="s">
         <v>1255</v>
       </c>
-      <c r="C393" s="239"/>
+      <c r="C393" s="238"/>
       <c r="D393" s="186" t="s">
-        <v>45</v>
+        <v>1231</v>
       </c>
       <c r="E393" s="186" t="s">
-        <v>45</v>
+        <v>34</v>
       </c>
       <c r="G393" s="30" t="s">
-        <v>1252</v>
+        <v>1232</v>
+      </c>
+      <c r="I393" s="240" t="s">
+        <v>1586</v>
       </c>
     </row>
     <row r="394" spans="2:12" ht="18" customHeight="1">
@@ -16200,584 +16248,641 @@
       </c>
       <c r="C394" s="239"/>
       <c r="D394" s="186" t="s">
-        <v>45</v>
+        <v>1231</v>
       </c>
       <c r="E394" s="186" t="s">
-        <v>45</v>
+        <v>357</v>
+      </c>
+      <c r="F394" s="92">
+        <v>24563</v>
       </c>
       <c r="G394" s="30" t="s">
-        <v>1252</v>
+        <v>1587</v>
+      </c>
+      <c r="I394" s="240" t="s">
+        <v>1593</v>
+      </c>
+      <c r="L394" s="240" t="s">
+        <v>1588</v>
       </c>
     </row>
     <row r="395" spans="2:12" ht="18" customHeight="1">
       <c r="B395" s="239" t="s">
-        <v>1257</v>
+        <v>1256</v>
       </c>
       <c r="C395" s="239"/>
       <c r="D395" s="186" t="s">
-        <v>45</v>
+        <v>1590</v>
       </c>
       <c r="E395" s="186" t="s">
-        <v>45</v>
+        <v>248</v>
+      </c>
+      <c r="F395" s="92">
+        <v>29552</v>
       </c>
       <c r="G395" s="30" t="s">
-        <v>1252</v>
+        <v>1589</v>
+      </c>
+      <c r="I395" s="240" t="s">
+        <v>1593</v>
+      </c>
+      <c r="L395" s="240" t="s">
+        <v>1588</v>
       </c>
     </row>
     <row r="396" spans="2:12" ht="18" customHeight="1">
       <c r="B396" s="239" t="s">
-        <v>1258</v>
+        <v>1256</v>
       </c>
       <c r="C396" s="239"/>
       <c r="D396" s="186" t="s">
+        <v>1231</v>
+      </c>
+      <c r="E396" s="186" t="s">
+        <v>1591</v>
+      </c>
+      <c r="F396" s="92">
+        <v>36123</v>
+      </c>
+      <c r="G396" s="30" t="s">
+        <v>1592</v>
+      </c>
+      <c r="I396" s="240" t="s">
+        <v>1593</v>
+      </c>
+      <c r="L396" s="240" t="s">
+        <v>1588</v>
+      </c>
+    </row>
+    <row r="397" spans="2:12" ht="18" customHeight="1">
+      <c r="B397" s="239" t="s">
+        <v>1257</v>
+      </c>
+      <c r="C397" s="239"/>
+      <c r="D397" s="186" t="s">
         <v>45</v>
       </c>
-      <c r="E396" s="186" t="s">
+      <c r="E397" s="186" t="s">
         <v>45</v>
       </c>
-      <c r="G396" s="30" t="s">
+      <c r="G397" s="30" t="s">
         <v>1252</v>
       </c>
     </row>
-    <row r="397" spans="2:12" ht="18" customHeight="1">
-      <c r="B397" s="201"/>
-      <c r="C397" s="201"/>
-      <c r="D397" s="159"/>
-      <c r="E397" s="159"/>
-      <c r="G397" s="30"/>
-    </row>
     <row r="398" spans="2:12" ht="18" customHeight="1">
-      <c r="B398" s="234" t="s">
-        <v>1259</v>
-      </c>
-      <c r="C398" s="234"/>
-      <c r="D398" s="177" t="s">
-        <v>176</v>
-      </c>
-      <c r="E398" s="177" t="s">
-        <v>34</v>
+      <c r="B398" s="239" t="s">
+        <v>1258</v>
+      </c>
+      <c r="C398" s="239"/>
+      <c r="D398" s="186" t="s">
+        <v>45</v>
+      </c>
+      <c r="E398" s="186" t="s">
+        <v>45</v>
       </c>
       <c r="G398" s="30" t="s">
-        <v>1260</v>
-      </c>
-      <c r="I398" s="240" t="s">
-        <v>1261</v>
+        <v>1252</v>
       </c>
     </row>
     <row r="399" spans="2:12" ht="18" customHeight="1">
-      <c r="B399" s="234" t="s">
-        <v>1262</v>
-      </c>
-      <c r="C399" s="234"/>
-      <c r="D399" s="177" t="s">
-        <v>25</v>
-      </c>
-      <c r="E399" s="177" t="s">
-        <v>26</v>
-      </c>
-      <c r="F399" s="35" t="s">
-        <v>1263</v>
-      </c>
-      <c r="G399" s="30" t="s">
-        <v>1264</v>
-      </c>
-      <c r="H399" s="26" t="s">
-        <v>724</v>
-      </c>
-      <c r="I399" s="240" t="s">
-        <v>1265</v>
-      </c>
-      <c r="J399" t="s">
-        <v>1266</v>
-      </c>
-      <c r="K399" t="s">
-        <v>1267</v>
-      </c>
+      <c r="B399" s="201"/>
+      <c r="C399" s="201"/>
+      <c r="D399" s="159"/>
+      <c r="E399" s="159"/>
+      <c r="G399" s="30"/>
     </row>
     <row r="400" spans="2:12" ht="18" customHeight="1">
       <c r="B400" s="234" t="s">
-        <v>1268</v>
+        <v>1259</v>
       </c>
       <c r="C400" s="234"/>
       <c r="D400" s="177" t="s">
-        <v>356</v>
+        <v>176</v>
       </c>
       <c r="E400" s="177" t="s">
-        <v>62</v>
-      </c>
-      <c r="F400" s="92">
-        <v>9051</v>
+        <v>34</v>
       </c>
       <c r="G400" s="30" t="s">
-        <v>1269</v>
-      </c>
-      <c r="H400" s="26" t="s">
-        <v>1270</v>
+        <v>1260</v>
       </c>
       <c r="I400" s="240" t="s">
-        <v>1271</v>
-      </c>
-      <c r="J400" s="1" t="s">
-        <v>1272</v>
-      </c>
-      <c r="K400" s="191" t="s">
-        <v>1273</v>
-      </c>
-      <c r="L400" s="240" t="s">
-        <v>1274</v>
+        <v>1261</v>
       </c>
     </row>
     <row r="401" spans="2:13" ht="18" customHeight="1">
       <c r="B401" s="234" t="s">
-        <v>1275</v>
+        <v>1262</v>
       </c>
       <c r="C401" s="234"/>
       <c r="D401" s="177" t="s">
+        <v>25</v>
+      </c>
+      <c r="E401" s="177" t="s">
+        <v>26</v>
+      </c>
+      <c r="F401" s="35" t="s">
+        <v>1263</v>
+      </c>
+      <c r="G401" s="30" t="s">
+        <v>1264</v>
+      </c>
+      <c r="H401" s="26" t="s">
+        <v>724</v>
+      </c>
+      <c r="I401" s="240" t="s">
+        <v>1265</v>
+      </c>
+      <c r="J401" t="s">
+        <v>1266</v>
+      </c>
+      <c r="K401" t="s">
+        <v>1267</v>
+      </c>
+    </row>
+    <row r="402" spans="2:13" ht="18" customHeight="1">
+      <c r="B402" s="234" t="s">
+        <v>1268</v>
+      </c>
+      <c r="C402" s="234"/>
+      <c r="D402" s="177" t="s">
+        <v>356</v>
+      </c>
+      <c r="E402" s="177" t="s">
+        <v>62</v>
+      </c>
+      <c r="F402" s="92">
+        <v>9051</v>
+      </c>
+      <c r="G402" s="30" t="s">
+        <v>1269</v>
+      </c>
+      <c r="H402" s="26" t="s">
+        <v>1270</v>
+      </c>
+      <c r="I402" s="240" t="s">
+        <v>1271</v>
+      </c>
+      <c r="J402" s="1" t="s">
+        <v>1272</v>
+      </c>
+      <c r="K402" s="191" t="s">
+        <v>1273</v>
+      </c>
+      <c r="L402" s="240" t="s">
+        <v>1274</v>
+      </c>
+    </row>
+    <row r="403" spans="2:13" ht="18" customHeight="1">
+      <c r="B403" s="234" t="s">
+        <v>1275</v>
+      </c>
+      <c r="C403" s="234"/>
+      <c r="D403" s="177" t="s">
         <v>202</v>
       </c>
-      <c r="E401" s="177" t="s">
+      <c r="E403" s="177" t="s">
         <v>62</v>
       </c>
-      <c r="F401" s="35">
+      <c r="F403" s="35">
         <v>1870</v>
       </c>
-      <c r="G401" s="30" t="s">
+      <c r="G403" s="30" t="s">
         <v>1276</v>
       </c>
-      <c r="H401" s="26" t="s">
+      <c r="H403" s="26" t="s">
         <v>421</v>
-      </c>
-      <c r="I401" s="240" t="s">
-        <v>1277</v>
-      </c>
-      <c r="L401" s="240" t="s">
-        <v>1278</v>
-      </c>
-    </row>
-    <row r="402" spans="2:13" ht="18" customHeight="1">
-      <c r="B402" s="225" t="s">
-        <v>1279</v>
-      </c>
-      <c r="C402" s="225"/>
-      <c r="D402" s="176" t="s">
-        <v>202</v>
-      </c>
-      <c r="E402" s="176" t="s">
-        <v>34</v>
-      </c>
-      <c r="F402" s="35">
-        <v>1879</v>
-      </c>
-      <c r="G402" s="30" t="s">
-        <v>1280</v>
-      </c>
-      <c r="I402" s="240" t="s">
-        <v>1277</v>
-      </c>
-      <c r="K402" s="11"/>
-      <c r="L402" s="240" t="s">
-        <v>1278</v>
-      </c>
-    </row>
-    <row r="403" spans="2:13" ht="18" customHeight="1">
-      <c r="B403" s="225" t="s">
-        <v>1279</v>
-      </c>
-      <c r="C403" s="225"/>
-      <c r="D403" s="176" t="s">
-        <v>202</v>
-      </c>
-      <c r="E403" s="176" t="s">
-        <v>284</v>
-      </c>
-      <c r="F403" s="35">
-        <v>1876</v>
-      </c>
-      <c r="G403" s="30" t="s">
-        <v>1281</v>
-      </c>
-      <c r="H403" s="26" t="s">
-        <v>1282</v>
       </c>
       <c r="I403" s="240" t="s">
         <v>1277</v>
       </c>
-      <c r="K403" s="11" t="s">
-        <v>1283</v>
-      </c>
       <c r="L403" s="240" t="s">
         <v>1278</v>
       </c>
     </row>
     <row r="404" spans="2:13" ht="18" customHeight="1">
       <c r="B404" s="225" t="s">
-        <v>1284</v>
+        <v>1279</v>
       </c>
       <c r="C404" s="225"/>
       <c r="D404" s="176" t="s">
-        <v>1285</v>
+        <v>202</v>
       </c>
       <c r="E404" s="176" t="s">
-        <v>673</v>
-      </c>
-      <c r="F404" s="48"/>
+        <v>34</v>
+      </c>
+      <c r="F404" s="35">
+        <v>1879</v>
+      </c>
       <c r="G404" s="30" t="s">
-        <v>1286</v>
-      </c>
-      <c r="H404" s="44"/>
-      <c r="I404" s="246" t="s">
-        <v>1287</v>
-      </c>
-      <c r="K404" s="5"/>
+        <v>1280</v>
+      </c>
+      <c r="I404" s="240" t="s">
+        <v>1277</v>
+      </c>
+      <c r="K404" s="11"/>
+      <c r="L404" s="240" t="s">
+        <v>1278</v>
+      </c>
     </row>
     <row r="405" spans="2:13" ht="18" customHeight="1">
       <c r="B405" s="225" t="s">
-        <v>1288</v>
+        <v>1279</v>
       </c>
       <c r="C405" s="225"/>
       <c r="D405" s="176" t="s">
-        <v>1289</v>
+        <v>202</v>
       </c>
       <c r="E405" s="176" t="s">
-        <v>43</v>
-      </c>
-      <c r="F405" s="91">
-        <v>1824</v>
+        <v>284</v>
+      </c>
+      <c r="F405" s="35">
+        <v>1876</v>
       </c>
       <c r="G405" s="30" t="s">
-        <v>1290</v>
-      </c>
-      <c r="H405" s="44"/>
-      <c r="I405" s="246" t="s">
-        <v>1291</v>
-      </c>
-      <c r="J405" t="s">
-        <v>1292</v>
-      </c>
-      <c r="K405" s="5"/>
+        <v>1281</v>
+      </c>
+      <c r="H405" s="26" t="s">
+        <v>1282</v>
+      </c>
+      <c r="I405" s="240" t="s">
+        <v>1277</v>
+      </c>
+      <c r="K405" s="11" t="s">
+        <v>1283</v>
+      </c>
       <c r="L405" s="240" t="s">
-        <v>1293</v>
+        <v>1278</v>
       </c>
     </row>
     <row r="406" spans="2:13" ht="18" customHeight="1">
       <c r="B406" s="225" t="s">
-        <v>1288</v>
+        <v>1284</v>
       </c>
       <c r="C406" s="225"/>
       <c r="D406" s="176" t="s">
+        <v>1285</v>
+      </c>
+      <c r="E406" s="176" t="s">
+        <v>673</v>
+      </c>
+      <c r="F406" s="48"/>
+      <c r="G406" s="30" t="s">
+        <v>1286</v>
+      </c>
+      <c r="H406" s="44"/>
+      <c r="I406" s="246" t="s">
+        <v>1287</v>
+      </c>
+      <c r="K406" s="5"/>
+    </row>
+    <row r="407" spans="2:13" ht="18" customHeight="1">
+      <c r="B407" s="225" t="s">
+        <v>1288</v>
+      </c>
+      <c r="C407" s="225"/>
+      <c r="D407" s="176" t="s">
         <v>1289</v>
       </c>
-      <c r="E406" s="176" t="s">
+      <c r="E407" s="176" t="s">
+        <v>43</v>
+      </c>
+      <c r="F407" s="91">
+        <v>1824</v>
+      </c>
+      <c r="G407" s="30" t="s">
+        <v>1290</v>
+      </c>
+      <c r="H407" s="44"/>
+      <c r="I407" s="246" t="s">
+        <v>1291</v>
+      </c>
+      <c r="J407" t="s">
+        <v>1292</v>
+      </c>
+      <c r="K407" s="5"/>
+      <c r="L407" s="240" t="s">
+        <v>1293</v>
+      </c>
+    </row>
+    <row r="408" spans="2:13" ht="18" customHeight="1">
+      <c r="B408" s="225" t="s">
+        <v>1288</v>
+      </c>
+      <c r="C408" s="225"/>
+      <c r="D408" s="176" t="s">
+        <v>1289</v>
+      </c>
+      <c r="E408" s="176" t="s">
         <v>34</v>
       </c>
-      <c r="F406" s="91" t="s">
+      <c r="F408" s="91" t="s">
         <v>1294</v>
       </c>
-      <c r="G406" s="30" t="s">
+      <c r="G408" s="30" t="s">
         <v>1290</v>
       </c>
-      <c r="H406" s="44" t="s">
+      <c r="H408" s="44" t="s">
         <v>761</v>
       </c>
-      <c r="I406" s="246" t="s">
+      <c r="I408" s="246" t="s">
         <v>1291</v>
       </c>
-      <c r="J406" t="s">
+      <c r="J408" t="s">
         <v>1292</v>
       </c>
-      <c r="K406" s="5"/>
-      <c r="L406" s="240" t="s">
+      <c r="K408" s="5"/>
+      <c r="L408" s="240" t="s">
         <v>1293</v>
       </c>
     </row>
-    <row r="407" spans="2:13" ht="18" customHeight="1">
-      <c r="B407" s="216"/>
-      <c r="C407" s="216"/>
-      <c r="D407" s="170"/>
-      <c r="E407" s="170"/>
-      <c r="F407" s="91"/>
-      <c r="G407" s="42"/>
-      <c r="H407" s="44"/>
-      <c r="I407" s="246"/>
-      <c r="K407" s="5"/>
-    </row>
-    <row r="408" spans="2:13" ht="18" customHeight="1">
-      <c r="B408" s="203" t="s">
+    <row r="409" spans="2:13" ht="18" customHeight="1">
+      <c r="B409" s="216"/>
+      <c r="C409" s="216"/>
+      <c r="D409" s="170"/>
+      <c r="E409" s="170"/>
+      <c r="F409" s="91"/>
+      <c r="G409" s="42"/>
+      <c r="H409" s="44"/>
+      <c r="I409" s="246"/>
+      <c r="K409" s="5"/>
+    </row>
+    <row r="410" spans="2:13" ht="18" customHeight="1">
+      <c r="B410" s="203" t="s">
         <v>1295</v>
       </c>
-      <c r="C408" s="203"/>
-      <c r="D408" s="161" t="s">
+      <c r="C410" s="203"/>
+      <c r="D410" s="161" t="s">
         <v>283</v>
       </c>
-      <c r="E408" s="161" t="s">
+      <c r="E410" s="161" t="s">
         <v>26</v>
       </c>
-      <c r="F408" s="35" t="s">
+      <c r="F410" s="35" t="s">
         <v>1296</v>
       </c>
-      <c r="G408" s="30" t="s">
+      <c r="G410" s="30" t="s">
         <v>1297</v>
       </c>
-      <c r="H408" s="26">
+      <c r="H410" s="26">
         <v>87</v>
       </c>
-      <c r="I408" s="240" t="s">
+      <c r="I410" s="240" t="s">
         <v>1298</v>
       </c>
-      <c r="J408" s="1" t="s">
+      <c r="J410" s="1" t="s">
         <v>156</v>
       </c>
-      <c r="K408" t="s">
+      <c r="K410" t="s">
         <v>1299</v>
       </c>
-      <c r="L408" s="240" t="s">
+      <c r="L410" s="240" t="s">
         <v>1300</v>
-      </c>
-    </row>
-    <row r="409" spans="2:13" ht="18" customHeight="1">
-      <c r="B409" s="203" t="s">
-        <v>1301</v>
-      </c>
-      <c r="C409" s="203"/>
-      <c r="D409" s="161" t="s">
-        <v>283</v>
-      </c>
-      <c r="E409" s="161" t="s">
-        <v>26</v>
-      </c>
-      <c r="F409" s="35" t="s">
-        <v>1302</v>
-      </c>
-      <c r="G409" s="30" t="s">
-        <v>1297</v>
-      </c>
-      <c r="H409" s="26"/>
-      <c r="I409" s="240" t="s">
-        <v>1298</v>
-      </c>
-      <c r="J409" s="1"/>
-      <c r="L409" s="240" t="s">
-        <v>1300</v>
-      </c>
-    </row>
-    <row r="410" spans="2:13" ht="18" customHeight="1">
-      <c r="B410" s="204" t="s">
-        <v>1303</v>
-      </c>
-      <c r="C410" s="204"/>
-      <c r="D410" s="160" t="s">
-        <v>51</v>
-      </c>
-      <c r="E410" s="160" t="s">
-        <v>248</v>
-      </c>
-      <c r="F410" s="35" t="s">
-        <v>1304</v>
-      </c>
-      <c r="G410" s="30" t="s">
-        <v>1305</v>
-      </c>
-      <c r="H410" s="26" t="s">
-        <v>315</v>
-      </c>
-      <c r="I410" s="240" t="s">
-        <v>1306</v>
-      </c>
-      <c r="K410" t="s">
-        <v>1307</v>
-      </c>
-      <c r="L410" s="240" t="s">
-        <v>1308</v>
       </c>
     </row>
     <row r="411" spans="2:13" ht="18" customHeight="1">
       <c r="B411" s="203" t="s">
-        <v>1309</v>
+        <v>1301</v>
       </c>
       <c r="C411" s="203"/>
       <c r="D411" s="161" t="s">
+        <v>283</v>
+      </c>
+      <c r="E411" s="161" t="s">
+        <v>26</v>
+      </c>
+      <c r="F411" s="35" t="s">
+        <v>1302</v>
+      </c>
+      <c r="G411" s="30" t="s">
+        <v>1297</v>
+      </c>
+      <c r="H411" s="26"/>
+      <c r="I411" s="240" t="s">
+        <v>1298</v>
+      </c>
+      <c r="J411" s="1"/>
+      <c r="L411" s="240" t="s">
+        <v>1300</v>
+      </c>
+    </row>
+    <row r="412" spans="2:13" ht="18" customHeight="1">
+      <c r="B412" s="204" t="s">
+        <v>1303</v>
+      </c>
+      <c r="C412" s="204"/>
+      <c r="D412" s="160" t="s">
+        <v>51</v>
+      </c>
+      <c r="E412" s="160" t="s">
+        <v>248</v>
+      </c>
+      <c r="F412" s="35" t="s">
+        <v>1304</v>
+      </c>
+      <c r="G412" s="30" t="s">
+        <v>1305</v>
+      </c>
+      <c r="H412" s="26" t="s">
+        <v>315</v>
+      </c>
+      <c r="I412" s="240" t="s">
+        <v>1306</v>
+      </c>
+      <c r="K412" t="s">
+        <v>1307</v>
+      </c>
+      <c r="L412" s="240" t="s">
+        <v>1308</v>
+      </c>
+    </row>
+    <row r="413" spans="2:13" ht="18" customHeight="1">
+      <c r="B413" s="203" t="s">
+        <v>1309</v>
+      </c>
+      <c r="C413" s="203"/>
+      <c r="D413" s="161" t="s">
         <v>604</v>
       </c>
-      <c r="E411" s="161" t="s">
+      <c r="E413" s="161" t="s">
         <v>673</v>
       </c>
-      <c r="G411" s="30" t="s">
+      <c r="G413" s="30" t="s">
         <v>1310</v>
       </c>
-      <c r="I411" t="s">
+      <c r="I413" t="s">
         <v>1311</v>
       </c>
-      <c r="K411" t="s">
+      <c r="K413" t="s">
         <v>1307</v>
       </c>
-      <c r="L411" s="240" t="s">
+      <c r="L413" s="240" t="s">
         <v>1312</v>
       </c>
     </row>
-    <row r="412" spans="2:13" ht="18" customHeight="1">
-      <c r="B412" s="203" t="s">
+    <row r="414" spans="2:13" ht="18" customHeight="1">
+      <c r="B414" s="203" t="s">
         <v>1313</v>
       </c>
-      <c r="C412" s="203"/>
-      <c r="D412" s="161" t="s">
+      <c r="C414" s="203"/>
+      <c r="D414" s="161" t="s">
         <v>604</v>
       </c>
-      <c r="E412" s="161" t="s">
+      <c r="E414" s="161" t="s">
         <v>26</v>
       </c>
-      <c r="F412" s="35" t="s">
+      <c r="F414" s="35" t="s">
         <v>1314</v>
       </c>
-      <c r="G412" s="30" t="s">
+      <c r="G414" s="30" t="s">
         <v>1315</v>
       </c>
-      <c r="H412" s="26">
+      <c r="H414" s="26">
         <v>98</v>
       </c>
-      <c r="I412" t="s">
+      <c r="I414" t="s">
         <v>1311</v>
       </c>
-      <c r="J412" s="1"/>
-      <c r="L412" s="240" t="s">
+      <c r="J414" s="1"/>
+      <c r="L414" s="240" t="s">
         <v>1312</v>
       </c>
     </row>
-    <row r="413" spans="2:13" s="5" customFormat="1" ht="18" customHeight="1">
-      <c r="B413" s="274" t="s">
+    <row r="415" spans="2:13" s="5" customFormat="1" ht="18" customHeight="1">
+      <c r="B415" s="274" t="s">
         <v>1313</v>
       </c>
-      <c r="C413" s="274"/>
-      <c r="D413" s="187" t="s">
+      <c r="C415" s="274"/>
+      <c r="D415" s="187" t="s">
         <v>604</v>
       </c>
-      <c r="E413" s="187" t="s">
+      <c r="E415" s="187" t="s">
         <v>143</v>
       </c>
-      <c r="F413" s="44" t="s">
+      <c r="F415" s="44" t="s">
         <v>1316</v>
       </c>
-      <c r="G413" s="44" t="s">
+      <c r="G415" s="44" t="s">
         <v>1317</v>
       </c>
-      <c r="H413" s="48" t="s">
+      <c r="H415" s="48" t="s">
         <v>1318</v>
       </c>
-      <c r="I413" s="246" t="s">
+      <c r="I415" s="246" t="s">
         <v>1311</v>
       </c>
-      <c r="K413" s="5" t="s">
+      <c r="K415" s="5" t="s">
         <v>1319</v>
       </c>
-      <c r="L413" s="246" t="s">
+      <c r="L415" s="246" t="s">
         <v>1320</v>
       </c>
-      <c r="M413" s="5" t="s">
+      <c r="M415" s="5" t="s">
         <v>1321</v>
       </c>
     </row>
-    <row r="414" spans="2:13" s="5" customFormat="1" ht="18" customHeight="1">
-      <c r="B414" s="274" t="s">
+    <row r="416" spans="2:13" s="5" customFormat="1" ht="18" customHeight="1">
+      <c r="B416" s="274" t="s">
         <v>1313</v>
       </c>
-      <c r="C414" s="274"/>
-      <c r="D414" s="187" t="s">
+      <c r="C416" s="274"/>
+      <c r="D416" s="187" t="s">
         <v>604</v>
       </c>
-      <c r="E414" s="187" t="s">
+      <c r="E416" s="187" t="s">
         <v>446</v>
       </c>
-      <c r="F414" s="44" t="s">
+      <c r="F416" s="44" t="s">
         <v>1322</v>
       </c>
-      <c r="G414" s="44" t="s">
+      <c r="G416" s="44" t="s">
         <v>1323</v>
       </c>
-      <c r="H414" s="48">
+      <c r="H416" s="48">
         <v>96</v>
       </c>
-      <c r="I414" s="246" t="s">
+      <c r="I416" s="246" t="s">
         <v>1311</v>
       </c>
-      <c r="L414" s="246" t="s">
+      <c r="L416" s="246" t="s">
         <v>1320</v>
-      </c>
-    </row>
-    <row r="415" spans="2:13" ht="18" customHeight="1">
-      <c r="B415" s="203" t="s">
-        <v>1324</v>
-      </c>
-      <c r="C415" s="203" t="s">
-        <v>107</v>
-      </c>
-      <c r="D415" s="161" t="s">
-        <v>604</v>
-      </c>
-      <c r="E415" s="161" t="s">
-        <v>1325</v>
-      </c>
-      <c r="G415" s="30" t="s">
-        <v>1326</v>
-      </c>
-    </row>
-    <row r="416" spans="2:13" ht="18" customHeight="1">
-      <c r="B416" s="203" t="s">
-        <v>1327</v>
-      </c>
-      <c r="C416" s="203"/>
-      <c r="D416" s="161" t="s">
-        <v>604</v>
-      </c>
-      <c r="E416" s="161" t="s">
-        <v>62</v>
-      </c>
-      <c r="G416" s="30" t="s">
-        <v>1328</v>
-      </c>
-      <c r="H416" s="26" t="s">
-        <v>233</v>
-      </c>
-      <c r="I416" t="s">
-        <v>1329</v>
       </c>
     </row>
     <row r="417" spans="2:12" ht="18" customHeight="1">
       <c r="B417" s="203" t="s">
+        <v>1324</v>
+      </c>
+      <c r="C417" s="203" t="s">
+        <v>107</v>
+      </c>
+      <c r="D417" s="161" t="s">
+        <v>604</v>
+      </c>
+      <c r="E417" s="161" t="s">
+        <v>1325</v>
+      </c>
+      <c r="G417" s="30" t="s">
+        <v>1326</v>
+      </c>
+    </row>
+    <row r="418" spans="2:12" ht="18" customHeight="1">
+      <c r="B418" s="203" t="s">
+        <v>1327</v>
+      </c>
+      <c r="C418" s="203"/>
+      <c r="D418" s="161" t="s">
+        <v>604</v>
+      </c>
+      <c r="E418" s="161" t="s">
+        <v>62</v>
+      </c>
+      <c r="G418" s="30" t="s">
+        <v>1328</v>
+      </c>
+      <c r="H418" s="26" t="s">
+        <v>233</v>
+      </c>
+      <c r="I418" t="s">
+        <v>1329</v>
+      </c>
+    </row>
+    <row r="419" spans="2:12" ht="18" customHeight="1">
+      <c r="B419" s="203" t="s">
         <v>1330</v>
       </c>
-      <c r="C417" s="203"/>
-      <c r="D417" s="161" t="s">
+      <c r="C419" s="203"/>
+      <c r="D419" s="161" t="s">
         <v>1331</v>
       </c>
-      <c r="E417" s="161" t="s">
+      <c r="E419" s="161" t="s">
         <v>1332</v>
       </c>
-      <c r="F417" s="35" t="s">
+      <c r="F419" s="35" t="s">
         <v>1333</v>
       </c>
-      <c r="G417" s="30" t="s">
+      <c r="G419" s="30" t="s">
         <v>1334</v>
       </c>
-      <c r="H417" s="26" t="s">
+      <c r="H419" s="26" t="s">
         <v>196</v>
       </c>
-      <c r="J417" s="1"/>
-      <c r="L417" s="240" t="s">
+      <c r="J419" s="1"/>
+      <c r="L419" s="240" t="s">
         <v>1335</v>
       </c>
     </row>
-    <row r="418" spans="2:12" ht="18" customHeight="1"/>
-    <row r="419" spans="2:12" ht="18" customHeight="1"/>
     <row r="420" spans="2:12" ht="18" customHeight="1"/>
-    <row r="449" spans="6:13">
-      <c r="F449" s="69"/>
-    </row>
-    <row r="452" spans="6:13">
-      <c r="K452" t="s">
+    <row r="421" spans="2:12" ht="18" customHeight="1"/>
+    <row r="422" spans="2:12" ht="18" customHeight="1"/>
+    <row r="451" spans="6:13">
+      <c r="F451" s="69"/>
+    </row>
+    <row r="454" spans="6:13">
+      <c r="K454" t="s">
         <v>1336</v>
       </c>
     </row>
-    <row r="462" spans="6:13">
-      <c r="M462" s="1"/>
+    <row r="464" spans="6:13">
+      <c r="M464" s="1"/>
     </row>
   </sheetData>
   <printOptions horizontalCentered="1" verticalCentered="1"/>

</xml_diff>

<commit_message>
Updates as per meeting with Cora
</commit_message>
<xml_diff>
--- a/assets/list/AD_Master_Data Base Templecurraheen Graveyard Feb23.xlsx
+++ b/assets/list/AD_Master_Data Base Templecurraheen Graveyard Feb23.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Templecurraheen\website\assets\list\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA7D897D-6FA8-4524-B183-300D35AAC493}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0321F34C-7282-47F5-BBA6-FF9BBC569EF2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="46296" windowHeight="25416" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3742" uniqueCount="1594">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3742" uniqueCount="1595">
   <si>
     <t>Mark</t>
   </si>
@@ -4804,6 +4804,9 @@
   </si>
   <si>
     <t>t156.jpg</t>
+  </si>
+  <si>
+    <t>Rev. John</t>
   </si>
 </sst>
 </file>
@@ -12250,7 +12253,7 @@
         <v>758</v>
       </c>
       <c r="E219" s="169" t="s">
-        <v>62</v>
+        <v>1594</v>
       </c>
       <c r="F219" s="35" t="s">
         <v>759</v>

</xml_diff>